<commit_message>
docs(rental-spec): simplify language to plain english and calibrate descriptive depth
</commit_message>
<xml_diff>
--- a/Rental Final Table/LetzRyd_Rental_Engine_Master_Specification.xlsx
+++ b/Rental Final Table/LetzRyd_Rental_Engine_Master_Specification.xlsx
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="₹#,##0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,13 +40,13 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="000F2537"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Consolas"/>
@@ -56,7 +56,7 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="001A1A1A"/>
+      <color rgb="00222222"/>
       <sz val="9"/>
     </font>
     <font>
@@ -69,12 +69,6 @@
       <name val="Segoe UI"/>
       <color rgb="00333333"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="000F2537"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="8">
@@ -116,8 +110,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
-        <bgColor rgb="00DDEBF7"/>
+        <fgColor rgb="00EBF1F5"/>
+        <bgColor rgb="00EBF1F5"/>
       </patternFill>
     </fill>
   </fills>
@@ -147,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -184,10 +178,16 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -570,15 +570,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:F17"/>
+  <dimension ref="A2:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -592,7 +591,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>1. Core Tables Summary</t>
+          <t>1. Summary of the 5 Tables</t>
         </is>
       </c>
     </row>
@@ -604,27 +603,22 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Type / Layer</t>
+          <t>Where it Comes From</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Records</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Records</t>
+          <t>What it Does (In Simple Words)</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>What This Table Is Used For</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Key Role in Engine</t>
+          <t>Why We Need It</t>
         </is>
       </c>
     </row>
@@ -636,27 +630,22 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Sheet Staging (Catalog)</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Google Sheet (Rental Slab tabs)</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>54 active tiers</t>
+          <t>Rental Slab tabs in Google Sheet</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>54 rows</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>This is the official price menu. It lists the daily rent for each trip target (e.g. 50-69 trips) for each city and car model.</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Stores the official pricing menu for all cities. Defines weekly trip brackets and daily base rents for each car model.</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Provides the rate card for standard Uber reducing plans and standard All-Platform flat plans.</t>
+          <t>The system checks this to find what rent a driver earned from their weekly trips.</t>
         </is>
       </c>
     </row>
@@ -668,27 +657,22 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Sheet Staging (Agreements)</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Google Sheet (Driver platform tabs)</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>511 partner deals</t>
+          <t>Driver Platform tabs in Google Sheet</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>511 rows</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Lists all drivers and fleet operators, their chosen plan (Uber or All-Platform), and any special discount rates.</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>Stores driver agreements, platform types, and special negotiated deals for fleet operators.</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>Identifies who has a custom negotiated rate (e.g. ₹970 or ₹1,070) or reduced indemnity (e.g. ₹15 or ₹0).</t>
+          <t>The system checks this to see if an operator has a negotiated deal (like ₹970 or ₹1,070/day).</t>
         </is>
       </c>
     </row>
@@ -700,27 +684,22 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Master Contract Table</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Allocations + sheet_rental_partners</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>1,512 contracts</t>
+          <t>Created from vehicle assignments</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>1,512 rows</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>The active contract for each car. It links the car number to the driver, their daily rent, and their daily insurance fee.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>The legal master agreement for every vehicle. Binds the vehicle, driver/operator, plan type, custom daily rent, and daily indemnity.</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Single source of truth used by the calculation engine for daily billing.</t>
+          <t>This is the main table the system reads every day to calculate rent.</t>
         </is>
       </c>
     </row>
@@ -732,27 +711,22 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Audit Trail Table</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>Automatic Database Triggers</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>1,512+ audit logs</t>
+          <t>Automatically saved by the system</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>1,512+ rows</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>A permanent history log. Whenever someone changes a car's rent or plan, it records who changed it, when, and why.</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Immutable history of every contract change. Records old rate, new rate, effective date, change reason, and who made the change.</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>Ensures financial accountability and prevents unauthorized or untracked rate changes.</t>
+          <t>Stops mistakes and gives a clear record if there is any question about past rent.</t>
         </is>
       </c>
     </row>
@@ -764,109 +738,98 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Daily Settlement Ledger</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>core_rent + attendance + trips</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Daily ledger</t>
+          <t>Calculated daily by the system</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Daily rows</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>The daily bill for each car. Shows if the car was on the road, trips done, daily rent, and daily insurance fee.</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Calculates and stores daily rent for every vehicle based on attendance status, earned trip tier, and indemnity fees.</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>Produces the final weekly settlement (Hisaab) totals for driver wallets and operator payouts.</t>
+          <t>Used to make the weekly Hisaab settlement sheet every Sunday night.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2. Rental Calculation Formulas</t>
+          <t>2. How the Rent is Calculated (Simple Formulas)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>Daily Rent Formula</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Net Daily Rent = Applied Daily Rent + Applied Daily Indemnity</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="12" t="inlineStr">
-        <is>
-          <t>Calculated for each vehicle for every calendar day. If the vehicle is On-Road, both rent and indemnity are charged. If in workshop, both are ₹0.00.</t>
-        </is>
-      </c>
-      <c r="F15" s="11" t="n"/>
+          <t>Daily Rent</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Net Daily Rent = Car Rent + Insurance (Indemnity)</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Calculated for every active car each day. If the car is on the road, both rent and insurance apply. If in garage, both are ₹0.</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Weekly Settlement (Hisaab)</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="n"/>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Total Weekly Rent = (Applied Daily Rent × On-Road Days) + (Applied Daily Indemnity × On-Road Days)</t>
-        </is>
-      </c>
-      <c r="D16" s="11" t="n"/>
-      <c r="E16" s="12" t="inlineStr">
-        <is>
-          <t>Settled every Sunday at midnight. The driver's earned trip tier sets the daily rent, which multiplies only across active on-road days.</t>
-        </is>
-      </c>
-      <c r="F16" s="11" t="n"/>
+          <t>Weekly Total (Hisaab)</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Weekly Total = (Daily Rent × On-Road Days) + (Daily Insurance × On-Road Days)</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Settled every Sunday night. The rate earned from weekly trips multiplies only by the days the car was actually driven.</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>Non-Billable Days</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="n"/>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Net Daily Rent = ₹0.00 (Rent = ₹0.00, Indemnity = ₹0.00)</t>
-        </is>
-      </c>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="12" t="inlineStr">
-        <is>
-          <t>When attendance status is 'Maintenance', 'Accident', or 'Breakdown', the day is non-billable and no fees are charged.</t>
-        </is>
-      </c>
-      <c r="F17" s="11" t="n"/>
+          <t>Cars in Workshop</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Net Daily Rent = ₹0.00</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>If a car is broken down or in the workshop, rent is ₹0 and insurance is ₹0 for those days.</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A2:F3"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="C17:D17"/>
+  <mergeCells count="7">
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="A2:E3"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="D17:E17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -881,18 +844,18 @@
   <dimension ref="A2:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
     <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>LetzRyd Rental Calculation Flow &amp; Rules</t>
+          <t>Rental Rules &amp; Step-by-Step Priority Flow</t>
         </is>
       </c>
     </row>
@@ -900,29 +863,29 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>1. Priority Resolution Order (How the Engine Decides Rent)</t>
+          <t>1. How the System Chooses the Rent (The 3 Priority Steps)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Step / Priority</t>
+          <t>Step</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Plan Type</t>
+          <t>Priority Level</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>When It Is Checked</t>
+          <t>Question the System Asks</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>How It Determines Rent</t>
+          <t>What Happens If YES</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -939,135 +902,139 @@
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>Step 1: Priority 1</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Special Deal / Custom Agreement</t>
+          <t>Step 1</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Priority 1:
+Special Deal / Custom Agreement</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Checked FIRST. Triggers whenever the driver or operator has a negotiated rate written in sheet_rental_partners or core_rent.</t>
+          <t>Does this driver or fleet operator have a negotiated daily rent agreed with LetzRyd?</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Applies the custom daily rent directly. Completely bypasses standard trip slabs and platform menus.</t>
+          <t>YES: The system charges that agreed rate directly. It stops here. It does not check trip counts or standard rate cards.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>No trips needed. Rent stays fixed regardless of trip count.</t>
+          <t>No trips needed. Rent stays fixed at the agreed rate.</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Mohd Abdul Qadir: WagonR @ ₹970/day, Dzire @ ₹1,070/day. Shaik Kareem: Xcent @ ₹900/day.</t>
+          <t>Mohd Abdul Qadir: WagonR @ ₹970/day, Dzire @ ₹1,070/day. Shaik Kareem: Xcent @ ₹900/day. Gaadylo: WagonR @ ₹900/day.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
-        <is>
-          <t>Step 2A: Priority 2A</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>Standard All-Platform Plan</t>
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>Step 2A</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Priority 2A:
+Standard All-Platform Plan</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Checked SECOND if no custom deal exists, and driver is registered as 'All Platform'.</t>
+          <t>If no special deal: Is this driver registered on the 'All Platform' plan (allowed to drive for Ola, Rapido, and Uber)?</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>Driver can drive on Ola, Uber, and Rapido. Uses the fixed menu card rate from sheet_rental_slabs for that city and model.</t>
+          <t>YES: The system charges the standard fixed menu rate for that city and car (e.g. ₹1,050 for WagonR, ₹1,200 for Dzire). It stops here.</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>No trips needed. Non-Uber trips are not tracked, so rent is flat.</t>
+          <t>No trips needed. Non-Uber trips are not tracked, so the rate is flat.</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>Standard WagonR driver on All-Platform pays flat ₹1,050/day across BLR, HYD, and MUM.</t>
+          <t>A regular All-Platform driver in Hyderabad or Bangalore pays a flat ₹1,050/day regardless of how many trips they do.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>Step 2B: Priority 2B</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Standard Uber Reducing Plan</t>
+          <t>Step 2B</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>Priority 2B:
+Standard Uber Reducing Plan</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Checked SECOND if no custom deal exists, and driver is registered on 'Uber Reducing Rent'.</t>
+          <t>If no special deal: Is this driver on the standard 'Uber Reducing Rent' plan?</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Sums completed Uber trips for the week (Mon-Sun). Looks up sheet_rental_slabs for that city and model, applying the earned tier.</t>
+          <t>YES: The system counts all Uber trips done from Monday to Sunday. It matches their trip total to the rate card. More trips = lower rent.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>High dependency. Completing more Uber trips moves driver to a cheaper daily rate tier.</t>
+          <t>High trip dependency. Completing more trips moves the driver to a cheaper rate tier.</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>Bangalore WagonR: 0-54 trips = ₹1,050/day; 55-69 trips = ₹950/day; 70+ trips = ₹850/day.</t>
+          <t>Bangalore WagonR: 0-54 trips = ₹1,050/day. 55-69 trips = ₹950/day. 70+ trips = ₹850/day.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>Step 3: Priority 3</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>System Fallback Rate</t>
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>Step 3</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Priority 3:
+System Fallback Safe Rate</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Checked LAST as a safety net if no custom deal exists and no matching slab is found in sheet_rental_slabs.</t>
+          <t>If no deal and no matching slab is found in the sheet (e.g. new unmapped model or missing sync)?</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Applies default base rate so billing never crashes: WagonR = ₹1,050, Dzire = ₹1,200, EC3/Other = ₹1,400.</t>
+          <t>YES: The system applies the default base rate (WagonR ₹1,050, Dzire ₹1,200, EC3 ₹1,400) so the system never breaks or charges zero.</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>No trips needed. Prevents unbilled days or database errors.</t>
+          <t>No trips needed. Acts as a safety net.</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Unmapped vehicle model safely charges base model rate until ops assigns an official plan.</t>
+          <t>Safely bills the standard base price until operations updates the rate card in the Google Sheet.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2. City-Level Pricing &amp; Indemnity Rules</t>
+          <t>2. City-Level Pricing &amp; Insurance Rules</t>
         </is>
       </c>
     </row>
@@ -1079,27 +1046,27 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Supported Models</t>
+          <t>Car Models Used</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Standard Indemnity</t>
+          <t>Standard Insurance (Indemnity)</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Special Indemnity Exceptions</t>
+          <t>Special Exceptions</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>All-Platform Flat Rate</t>
+          <t>All-Platform Rate</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Operational Notes</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -1121,8 +1088,8 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Nisamudeen K P = ₹15.00/day
-Rishad P V = ₹20.00/day</t>
+          <t>Nisamudeen K P pays ₹15/day
+Rishad P V pays ₹20/day</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -1132,19 +1099,19 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Offers distinct rate cards for Individual drivers vs Operator Fleets based on trip thresholds.</t>
+          <t>Has separate rate tiers for individual drivers vs fleet operators.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>Hyderabad (HYD)</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Maruti Wagonr, Maruti Dzire, Hyundai Xcent (Retired), EC3</t>
+          <t>Maruti Wagonr, Maruti Dzire, EC3, Hyundai Xcent (Retired)</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -1154,8 +1121,8 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Retired Hyundai Xcent fleet = ₹0.00/day
-Shaik Kareem = ₹0.00/day</t>
+          <t>Retired Hyundai Xcent fleet pays ₹0/day
+Shaik Kareem pays ₹0/day</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -1166,7 +1133,7 @@
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>Extensive fleet operators with negotiated side-table rates overriding standard cards.</t>
+          <t>Many fleet operators have negotiated deals that override standard cards.</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1155,7 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Included in weekly hisaab settlement as 'Insurance Amount'</t>
+          <t>Added to settlement as 'Insurance Amount'</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
@@ -1198,26 +1165,26 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Operates primarily on WagonR CNG with 6 dynamic trip reducing tiers (0-49 to 130+).</t>
+          <t>6 trip-reducing tiers starting from 0-49 trips up to 130+ trips.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>3. Operational Safeguards &amp; Edge Cases</t>
+          <t>3. Common Situations &amp; How the System Handles Them</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Rule / Case</t>
+          <t>Situation</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Operational Scenario</t>
+          <t>What Happens in Real Life</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1227,95 +1194,95 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Business Benefit</t>
+          <t>Result</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="inlineStr">
-        <is>
-          <t>Multi-Car Operators</t>
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Operator with Multiple Cars</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>An operator runs 10+ vehicles across different models (e.g. WagonR and Dzire).</t>
+          <t>An operator runs both WagonR and Dzire cars.</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Each vehicle has its own contract row in core_rent tied to vehicle_number. Slabs match both partner_id and vehicle_model.</t>
+          <t>Each car has its own record in core_rent. The system matches both the operator ID and the car model.</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Operator is billed accurately per model (e.g. Qadir Dzire = ₹1,070, WagonR = ₹970) with no rate mix-ups.</t>
+          <t>Dzires are charged Dzire rent (₹1,070) and WagonRs are charged WagonR rent (₹970). No mixing.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>Driver Moonlighting</t>
+          <t>Driver Moonlighting on Ola</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>An Uber driver splits time driving on Ola or Rapido.</t>
+          <t>A driver on the Uber plan spends time driving for Ola.</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>System only counts Uber trips. Untracked Ola trips keep Uber count low, placing driver in Tier 1 (₹1,050/day).</t>
+          <t>Only Uber trips are counted. Fewer Uber trips mean the driver stays in the lowest tier (0-49 trips).</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Company is protected: driver automatically loses discounts and pays full standard base rent.</t>
+          <t>Driver pays full base rent (₹1,050/day). The company is fully protected from revenue loss.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="inlineStr">
-        <is>
-          <t>Mid-Week Plan Freeze</t>
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>Mid-Week Plan Change</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Driver asks to switch from Uber Reducing to All-Platform on Wednesday.</t>
+          <t>A driver wants to switch plans on Wednesday.</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Rent does not fluctuate mid-week. Contract changes take effect the following Monday. Weekly settlement uses earned tier.</t>
+          <t>Rent stays locked until Sunday night. Plan changes only take effect starting next Monday.</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Eliminates confusion and disputes with drivers over mid-week recalculations.</t>
+          <t>Stops mid-week recalculation errors and billing disputes with drivers.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>Maintenance &amp; Garage</t>
+          <t>Car in Workshop / Breakdown</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Vehicle spends 2 days in the workshop for repairs.</t>
+          <t>A car is in the repair garage for 2 days during the week.</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Vehicle status is marked 'Maintenance' in sheet_vehicle_status. Engine sets is_billable_day = FALSE for those 2 days.</t>
+          <t>The daily status is marked 'Maintenance'. The system sets billable = FALSE for those 2 days.</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Driver is only billed for active on-road days (Rent = ₹0, Indemnity = ₹0 on workshop days).</t>
+          <t>Driver is charged ₹0 rent and ₹0 insurance for those 2 days.</t>
         </is>
       </c>
     </row>
@@ -1338,23 +1305,23 @@
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Database Schema &amp; Data Dictionary (5 Core Tables)</t>
+          <t>Database Schema &amp; Table Columns (In Plain English)</t>
         </is>
       </c>
     </row>
     <row r="3"/>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>Table 1: sheet_rental_slabs  (Google Sheet Staging Table (Syncs every 30 mins))</t>
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Table 1: sheet_rental_slabs  —  Google Sheet Rate Cards (Syncs every 30 minutes)</t>
         </is>
       </c>
       <c r="B5" s="11" t="n"/>
@@ -1363,10 +1330,10 @@
       <c r="E5" s="11" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>WHAT THIS TABLE IS USED FOR:
-This table is the official pricing menu synchronized from the live Google Sheet. It defines weekly trip tiers, daily base rents, and platform rules for each city and car model. The calculation engine queries this table to look up rate cards for standard Uber reducing plans and standard All-Platform plans.</t>
+This table is the official price menu copied from the Google Sheet. It stores the weekly trip targets and daily base rents for each city and car model. The system looks at this table to find the rate for standard Uber drivers and standard All-Platform drivers.</t>
         </is>
       </c>
       <c r="B6" s="11" t="n"/>
@@ -1394,17 +1361,17 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Constraints / Keys</t>
+          <t>Constraint</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Description &amp; Purpose (Plain English)</t>
+          <t>What This Column Stores (Simple English)</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Business Logic / Example Values</t>
+          <t>Example Value</t>
         </is>
       </c>
     </row>
@@ -1419,14 +1386,14 @@
           <t>SERIAL</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>PRIMARY KEY</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Unique numeric ID for each rate card tier.</t>
+          <t>Row number in the database.</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
@@ -1453,7 +1420,7 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Operating city where this rate card applies.</t>
+          <t>City where this price applies.</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -1480,7 +1447,7 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Vehicle model name matching vehicle onboarding records.</t>
+          <t>Car model name.</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -1507,7 +1474,7 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Fuel type specification of the vehicle.</t>
+          <t>Car fuel type.</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -1534,7 +1501,7 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>Uber operating plan type (TBS = Trip Based, EBS = Earnings Based).</t>
+          <t>Uber plan type (TBS = Trip Based, EBS = Earnings Based).</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -1561,7 +1528,7 @@
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Pricing category: 'Uber Reducing Rent' or 'All Platform'.</t>
+          <t>Plan name: 'Uber Reducing Rent' or 'All Platform'.</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1588,7 +1555,7 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Driver category in BLR: 'Individual' or 'Operator Fleet'.</t>
+          <t>Driver type in BLR: 'Individual' or 'Operator Fleet'.</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -1615,7 +1582,7 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>Human-readable label for the trip range.</t>
+          <t>Trip target label (e.g. 50-69 trips).</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1642,7 +1609,7 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Minimum completed trips needed to qualify for this rate.</t>
+          <t>Minimum trips needed for this price.</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -1669,7 +1636,7 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>Maximum trips for this tier (NULL for top open-ended tier).</t>
+          <t>Maximum trips for this price (empty for top tier).</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
@@ -1696,7 +1663,7 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Base daily rental fee charged to the driver.</t>
+          <t>Daily base rent for this trip tier.</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
@@ -1723,7 +1690,7 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Indemnity in rate card (standardized to 0.00; set in contract).</t>
+          <t>Indemnity in rate card (kept at 0; set in contract).</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
@@ -1750,7 +1717,7 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Target platform for this pricing tier.</t>
+          <t>Platform name for this slab.</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -1777,7 +1744,7 @@
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Whether extra platform trip bonuses pass to driver.</t>
+          <t>Whether extra Uber trip bonuses go to the driver.</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -1804,7 +1771,7 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Timestamp when this record was updated from Google Sheet.</t>
+          <t>When this row was last copied from Google Sheet.</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
@@ -1814,9 +1781,9 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="15" t="inlineStr">
-        <is>
-          <t>Table 2: sheet_rental_partners  (Google Sheet Staging Table (Syncs every 30 mins))</t>
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>Table 2: sheet_rental_partners  —  Google Sheet Driver &amp; Operator Agreements (Syncs every 30 minutes)</t>
         </is>
       </c>
       <c r="B27" s="11" t="n"/>
@@ -1825,10 +1792,10 @@
       <c r="E27" s="11" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
+      <c r="A28" s="18" t="inlineStr">
         <is>
           <t>WHAT THIS TABLE IS USED FOR:
-This table stores driver-partner agreements synced from the Google Sheet. It captures individual drivers, multi-car operators, platform bindings, custom negotiated flat daily rents, and special indemnity terms (like Nisamudeen ₹15, Shaik Kareem ₹0). Used during contract creation to resolve custom deals.</t>
+This table stores driver and fleet operator agreements copied from the Google Sheet. It lists who is on Uber vs All-Platform, who has a special negotiated daily rent (like ₹970), and who has a special insurance rate (like ₹15 or ₹0).</t>
         </is>
       </c>
       <c r="B28" s="11" t="n"/>
@@ -1856,17 +1823,17 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Constraints / Keys</t>
+          <t>Constraint</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Description &amp; Purpose (Plain English)</t>
+          <t>What This Column Stores (Simple English)</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Business Logic / Example Values</t>
+          <t>Example Value</t>
         </is>
       </c>
     </row>
@@ -1881,14 +1848,14 @@
           <t>VARCHAR(64)</t>
         </is>
       </c>
-      <c r="C31" s="14" t="inlineStr">
+      <c r="C31" s="15" t="inlineStr">
         <is>
           <t>PRIMARY KEY</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Unique partner identifier assigned during onboarding.</t>
+          <t>Unique partner ID code.</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -1915,7 +1882,7 @@
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>Full legal or commercial name of driver or fleet operator.</t>
+          <t>Full name of the driver or fleet operator.</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -1969,7 +1936,7 @@
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Partner classification: 'Individual' (1 car) or 'Operator Fleet' (multi-car).</t>
+          <t>Driver type: 'Individual' (1 car) or 'Operator Fleet' (multi-car).</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
@@ -1996,7 +1963,7 @@
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Agreed platform binding from onboarding.</t>
+          <t>Platform from onboarding.</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
@@ -2023,7 +1990,7 @@
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Settlement plan categorization used in hisaab sheets.</t>
+          <t>Plan category used in weekly hisaab.</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -2050,7 +2017,7 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Negotiated daily rent overriding standard rate cards.</t>
+          <t>Special agreed daily rent (empty if standard price applies).</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
@@ -2077,7 +2044,7 @@
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>Negotiated daily indemnity overriding standard ₹30 fee.</t>
+          <t>Special agreed daily insurance fee (empty if standard ₹30 applies).</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
@@ -2104,7 +2071,7 @@
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Operational remarks, vehicle models, or special contract conditions.</t>
+          <t>Extra notes about car models or special deal terms.</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
@@ -2131,7 +2098,7 @@
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>Timestamp when partner record was synced from Google Sheet.</t>
+          <t>When this row was last copied from Google Sheet.</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
@@ -2141,9 +2108,9 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="15" t="inlineStr">
-        <is>
-          <t>Table 3: core_rent  (Master Contract Table (PostgreSQL Master Agreement))</t>
+      <c r="A44" s="17" t="inlineStr">
+        <is>
+          <t>Table 3: core_rent  —  Main Contract Table (PostgreSQL Legal Agreements)</t>
         </is>
       </c>
       <c r="B44" s="11" t="n"/>
@@ -2152,10 +2119,10 @@
       <c r="E44" s="11" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="16" t="inlineStr">
+      <c r="A45" s="18" t="inlineStr">
         <is>
           <t>WHAT THIS TABLE IS USED FOR:
-This is the single source of truth for all vehicle rental contracts. It binds each vehicle registration number to an active partner, plan scheme, custom daily rent override, and daily indemnity fee. The daily calculation engine reads this table to determine what rules and rates apply to every vehicle.</t>
+This is the master contract table for every vehicle in the fleet. It links each car number to the driver, their plan, any special agreed rent, and their daily insurance fee. The daily billing system reads this table every day to know what to charge.</t>
         </is>
       </c>
       <c r="B45" s="11" t="n"/>
@@ -2183,17 +2150,17 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Constraints / Keys</t>
+          <t>Constraint</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Description &amp; Purpose (Plain English)</t>
+          <t>What This Column Stores (Simple English)</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Business Logic / Example Values</t>
+          <t>Example Value</t>
         </is>
       </c>
     </row>
@@ -2208,14 +2175,14 @@
           <t>SERIAL</t>
         </is>
       </c>
-      <c r="C48" s="14" t="inlineStr">
+      <c r="C48" s="15" t="inlineStr">
         <is>
           <t>PRIMARY KEY</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>Unique numeric identifier for each rental contract.</t>
+          <t>Contract serial number.</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
@@ -2242,7 +2209,7 @@
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>Official registration plate number of the vehicle.</t>
+          <t>Car registration plate number.</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
@@ -2269,7 +2236,7 @@
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Partner code holding the active agreement for this vehicle.</t>
+          <t>Partner ID code assigned to this car.</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
@@ -2296,7 +2263,7 @@
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>City where the vehicle is deployed.</t>
+          <t>City where the car is located.</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
@@ -2323,7 +2290,7 @@
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Vehicle model matching onboarding specifications.</t>
+          <t>Car model name.</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
@@ -2350,7 +2317,7 @@
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>Active plan scheme: 'Uber Reducing Rent' or 'All Platform Flat'.</t>
+          <t>Contract plan: 'Uber Reducing Rent' or 'All Platform Flat'.</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
@@ -2377,7 +2344,7 @@
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Priority 1 custom rent override. If set, bypasses trip slabs.</t>
+          <t>Special agreed daily rent (bypasses trip slabs if filled).</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
@@ -2404,7 +2371,7 @@
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Contractual daily indemnity fee charged for this vehicle.</t>
+          <t>Daily insurance fee charged for this car.</t>
         </is>
       </c>
       <c r="E55" s="6" t="inlineStr">
@@ -2431,7 +2398,7 @@
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Start date when this contract and pricing becomes active.</t>
+          <t>Date when this contract starts.</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
@@ -2458,7 +2425,7 @@
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>Expiry date when this contract ends.</t>
+          <t>Date when this contract ends.</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
@@ -2485,7 +2452,7 @@
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Whether this contract is currently active for daily billing.</t>
+          <t>Whether this contract is currently active.</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
@@ -2512,7 +2479,7 @@
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>System timestamp when contract record was created.</t>
+          <t>When this contract was first created.</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
@@ -2539,7 +2506,7 @@
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>System timestamp when contract was last modified.</t>
+          <t>When this contract was last updated.</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
@@ -2549,9 +2516,9 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="15" t="inlineStr">
-        <is>
-          <t>Table 4: core_rent_logs  (Audit Trail Table (Database Trigger-Driven))</t>
+      <c r="A64" s="17" t="inlineStr">
+        <is>
+          <t>Table 4: core_rent_logs  —  Audit History Log Table (Automatic)</t>
         </is>
       </c>
       <c r="B64" s="11" t="n"/>
@@ -2560,10 +2527,10 @@
       <c r="E64" s="11" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="16" t="inlineStr">
+      <c r="A65" s="18" t="inlineStr">
         <is>
           <t>WHAT THIS TABLE IS USED FOR:
-This is an append-only audit trail automatically populated by database triggers whenever core_rent is inserted, updated, or terminated. It records the old rate, new rate, effective timestamps, change reason, and who made the change. Ensures 100% financial compliance and contract change tracking.</t>
+This table keeps a permanent record of all contract changes. Whenever someone updates a car's rent or switches its plan, the system automatically writes a new row here with the old rate, the new rate, who changed it, and why.</t>
         </is>
       </c>
       <c r="B65" s="11" t="n"/>
@@ -2591,17 +2558,17 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Constraints / Keys</t>
+          <t>Constraint</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Description &amp; Purpose (Plain English)</t>
+          <t>What This Column Stores (Simple English)</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Business Logic / Example Values</t>
+          <t>Example Value</t>
         </is>
       </c>
     </row>
@@ -2616,14 +2583,14 @@
           <t>SERIAL</t>
         </is>
       </c>
-      <c r="C68" s="14" t="inlineStr">
+      <c r="C68" s="15" t="inlineStr">
         <is>
           <t>PRIMARY KEY</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Unique audit event log identifier.</t>
+          <t>Log event serial number.</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
@@ -2650,7 +2617,7 @@
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>Reference to the core_rent contract that was modified.</t>
+          <t>Contract ID that was changed.</t>
         </is>
       </c>
       <c r="E69" s="6" t="inlineStr">
@@ -2677,7 +2644,7 @@
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Registration number of the vehicle.</t>
+          <t>Car registration number.</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
@@ -2704,7 +2671,7 @@
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>Partner code associated with the contract.</t>
+          <t>Partner ID code on the contract.</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
@@ -2731,7 +2698,7 @@
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Previous plan scheme before the modification.</t>
+          <t>Previous plan before the change.</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
@@ -2758,7 +2725,7 @@
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>New plan scheme being activated.</t>
+          <t>New plan after the change.</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
@@ -2785,7 +2752,7 @@
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Previous custom daily rent before the update.</t>
+          <t>Previous daily rent before the update.</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
@@ -2812,7 +2779,7 @@
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>New custom daily rent assigned to the contract.</t>
+          <t>New daily rent after the update.</t>
         </is>
       </c>
       <c r="E75" s="6" t="inlineStr">
@@ -2839,7 +2806,7 @@
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Operational explanation for why the contract was modified.</t>
+          <t>Why the change was made.</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
@@ -2866,7 +2833,7 @@
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>User or background process that executed the modification.</t>
+          <t>Who made the change.</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
@@ -2893,7 +2860,7 @@
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Precise timestamp when the audit log was recorded.</t>
+          <t>Exact date and time when the change happened.</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
@@ -2903,9 +2870,9 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="15" t="inlineStr">
-        <is>
-          <t>Table 5: daily_rent_log  (Daily Settlement Ledger Table)</t>
+      <c r="A82" s="17" t="inlineStr">
+        <is>
+          <t>Table 5: daily_rent_log  —  Daily Billing Ledger (Production Daily Records)</t>
         </is>
       </c>
       <c r="B82" s="11" t="n"/>
@@ -2914,10 +2881,10 @@
       <c r="E82" s="11" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="16" t="inlineStr">
+      <c r="A83" s="18" t="inlineStr">
         <is>
           <t>WHAT THIS TABLE IS USED FOR:
-This table is the production daily billing ledger. For every vehicle on every calendar day, it records attendance status, whether the day is billable, completed weekly trips, applied daily rent, applied indemnity, and net daily rent. It is aggregated on Sunday to generate the weekly settlement (Hisaab).</t>
+This table is the daily billing record. Every day, it records whether each car was driven, weekly trips completed, the daily rent charged, and the daily insurance fee. At the end of the week, this data is summed up to make the driver's Hisaab payout.</t>
         </is>
       </c>
       <c r="B83" s="11" t="n"/>
@@ -2945,17 +2912,17 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Constraints / Keys</t>
+          <t>Constraint</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Description &amp; Purpose (Plain English)</t>
+          <t>What This Column Stores (Simple English)</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>Business Logic / Example Values</t>
+          <t>Example Value</t>
         </is>
       </c>
     </row>
@@ -2970,14 +2937,14 @@
           <t>BIGSERIAL</t>
         </is>
       </c>
-      <c r="C86" s="14" t="inlineStr">
+      <c r="C86" s="15" t="inlineStr">
         <is>
           <t>PRIMARY KEY</t>
         </is>
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>Unique transaction identifier for each daily ledger entry.</t>
+          <t>Daily transaction serial number.</t>
         </is>
       </c>
       <c r="E86" s="9" t="inlineStr">
@@ -3004,7 +2971,7 @@
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>Calendar date of the billing day.</t>
+          <t>Calendar date of this bill.</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
@@ -3031,7 +2998,7 @@
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>Settlement week identifier (e.g. 2026-W36: Mon to Sun).</t>
+          <t>Week identifier (e.g. 2026-W36: Mon to Sun).</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
@@ -3058,7 +3025,7 @@
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>Registration number of the vehicle.</t>
+          <t>Car registration number.</t>
         </is>
       </c>
       <c r="E89" s="4" t="inlineStr">
@@ -3085,7 +3052,7 @@
       </c>
       <c r="D90" s="9" t="inlineStr">
         <is>
-          <t>Partner responsible for this day's vehicle rental fees.</t>
+          <t>Partner responsible for this bill.</t>
         </is>
       </c>
       <c r="E90" s="7" t="inlineStr">
@@ -3112,7 +3079,7 @@
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>Operating city where vehicle is located.</t>
+          <t>City where the car is operated.</t>
         </is>
       </c>
       <c r="E91" s="4" t="inlineStr">
@@ -3139,7 +3106,7 @@
       </c>
       <c r="D92" s="9" t="inlineStr">
         <is>
-          <t>Vehicle model specifications.</t>
+          <t>Car model name.</t>
         </is>
       </c>
       <c r="E92" s="7" t="inlineStr">
@@ -3166,7 +3133,7 @@
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>Daily operational status ('On-Road', 'Maintenance', 'Breakdown').</t>
+          <t>Daily car status ('On-Road', 'Maintenance', 'Breakdown').</t>
         </is>
       </c>
       <c r="E93" s="4" t="inlineStr">
@@ -3193,7 +3160,7 @@
       </c>
       <c r="D94" s="9" t="inlineStr">
         <is>
-          <t>TRUE if status is On-Road; FALSE if in workshop (₹0 charged).</t>
+          <t>TRUE if car was on road; FALSE if in repair garage.</t>
         </is>
       </c>
       <c r="E94" s="9" t="inlineStr">
@@ -3220,7 +3187,7 @@
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>Cumulative completed weekly Uber trips for this week.</t>
+          <t>Total completed weekly Uber trips.</t>
         </is>
       </c>
       <c r="E95" s="6" t="inlineStr">
@@ -3247,7 +3214,7 @@
       </c>
       <c r="D96" s="9" t="inlineStr">
         <is>
-          <t>Daily base rent resolved by priority rules (₹0 if not billable).</t>
+          <t>Daily rent charged for this day (₹0 if in garage).</t>
         </is>
       </c>
       <c r="E96" s="9" t="inlineStr">
@@ -3274,7 +3241,7 @@
       </c>
       <c r="D97" s="6" t="inlineStr">
         <is>
-          <t>Daily indemnity fee resolved for this vehicle (₹0 if not billable).</t>
+          <t>Daily insurance charged for this day (₹0 if in garage).</t>
         </is>
       </c>
       <c r="E97" s="6" t="inlineStr">
@@ -3301,7 +3268,7 @@
       </c>
       <c r="D98" s="9" t="inlineStr">
         <is>
-          <t>Total billable daily fee = applied_daily_rent + applied_indemnity.</t>
+          <t>Total daily charge = daily rent + daily insurance.</t>
         </is>
       </c>
       <c r="E98" s="9" t="inlineStr">
@@ -3328,12 +3295,12 @@
       </c>
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>Audit trace explaining the exact pricing rule applied.</t>
+          <t>Short note explaining which rule was used.</t>
         </is>
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
-          <t>'Slab Tier: 70-89 (850.00/day)', 'Custom Deal: 970.00'</t>
+          <t>'Slab Tier: 70-89 (850/day)', 'Custom Deal: 970'</t>
         </is>
       </c>
     </row>
@@ -3364,24 +3331,24 @@
   <dimension ref="A2:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="46" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>LetzRyd Rental Calculation Scenarios &amp; Examples</t>
+          <t>Real Examples &amp; Calculations (In Simple Words)</t>
         </is>
       </c>
     </row>
@@ -3389,14 +3356,14 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>1. Walkthrough of Different Driver Plans &amp; Cases</t>
+          <t>1. Examples of Different Driver Cases</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Scenario / Driver Profile</t>
+          <t>Driver / Case</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -3406,12 +3373,12 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Vehicle Model</t>
+          <t>Car Model</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Plan Scheme</t>
+          <t>Plan Name</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -3421,44 +3388,44 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Days On-Road</t>
+          <t>Days Driven</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Priority Level Applied</t>
+          <t>Priority Step</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Applied Daily Rent (₹)</t>
+          <t>Daily Rent (₹)</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Daily Indemnity (₹)</t>
+          <t>Daily Insurance (₹)</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Net Daily Rent (₹)</t>
+          <t>Net Daily (₹)</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Total Weekly Rent (₹)</t>
+          <t>Weekly Total (₹)</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>Explanation &amp; Formula Used</t>
+          <t>Simple Explanation</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>1. High-Performance Uber Driver (Raju Sharma)</t>
+          <t>1. High-Trip Uber Driver (Raju)</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -3484,33 +3451,33 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Priority 2B (Uber Dynamic Slab)</t>
-        </is>
-      </c>
-      <c r="H7" s="17" t="n">
+          <t>Priority 2B (Uber Slab)</t>
+        </is>
+      </c>
+      <c r="H7" s="19" t="n">
         <v>850</v>
       </c>
-      <c r="I7" s="17" t="n">
+      <c r="I7" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="J7" s="18">
+      <c r="J7" s="20">
         <f>H7+I7</f>
         <v/>
       </c>
-      <c r="K7" s="18">
+      <c r="K7" s="20">
         <f>J7*F7</f>
         <v/>
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>Raju drove exclusively for Uber and hit 78 trips. Bangalore rate card assigns ₹850/day (tier 70+). With ₹30 indemnity, daily net = ₹880. Weekly total for 6 on-road days = 6 × ₹880 = ₹5,280.</t>
+          <t>Raju drove exclusively on Uber and did 78 trips. His high trips placed him in the 70+ tier (₹850/day). Net = ₹880/day. Weekly total for 6 days = ₹5,280.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>2. Moonlighting Driver on Ola (Suresh Kumar)</t>
+          <t>2. Moonlighting Driver on Ola (Suresh)</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -3536,33 +3503,33 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>Priority 2B (Uber Base Tier 1)</t>
-        </is>
-      </c>
-      <c r="H8" s="19" t="n">
+          <t>Priority 2B (Uber Tier 1)</t>
+        </is>
+      </c>
+      <c r="H8" s="21" t="n">
         <v>1050</v>
       </c>
-      <c r="I8" s="19" t="n">
+      <c r="I8" s="21" t="n">
         <v>30</v>
       </c>
-      <c r="J8" s="20">
+      <c r="J8" s="22">
         <f>H8+I8</f>
         <v/>
       </c>
-      <c r="K8" s="20">
+      <c r="K8" s="22">
         <f>J8*F8</f>
         <v/>
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Suresh is on an Uber contract but splits time driving for Ola. Untracked Ola trips leave his Uber count at only 24 trips. He stays in Tier 1 (₹1,050/day). Net daily = ₹1,080. Weekly total = ₹6,480. LetzRyd recovers full base rent.</t>
+          <t>Suresh is on an Uber plan but drove for Ola. With only 24 Uber trips recorded, he stays at base price (₹1,050/day). Net = ₹1,080/day. Weekly total = ₹6,480.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>3. Standard All-Platform Driver (Amit Patil)</t>
+          <t>3. All-Platform Driver (Amit)</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -3588,33 +3555,33 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Priority 2A (All-Platform Flat Slab)</t>
-        </is>
-      </c>
-      <c r="H9" s="17" t="n">
+          <t>Priority 2A (Flat Slab)</t>
+        </is>
+      </c>
+      <c r="H9" s="19" t="n">
         <v>1050</v>
       </c>
-      <c r="I9" s="17" t="n">
+      <c r="I9" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="J9" s="18">
+      <c r="J9" s="20">
         <f>H9+I9</f>
         <v/>
       </c>
-      <c r="K9" s="18">
+      <c r="K9" s="20">
         <f>J9*F9</f>
         <v/>
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>Amit signed an All-Platform contract with no custom deal. Trips are ignored. Engine applies standard All-Platform slab (₹1,050/day) + ₹30 indemnity = ₹1,080/day. Weekly total for 7 days = ₹7,560.</t>
+          <t>Amit drives for Ola, Uber, and Rapido. Trips are not counted. He pays flat menu rent of ₹1,050/day + ₹30 insurance = ₹1,080/day. Weekly total for 7 days = ₹7,560.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>4A. Multi-Car Operator - WagonR (Mohd Abdul Qadir)</t>
+          <t>4A. Fleet Operator - WagonR (Mohd Abdul Qadir)</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
@@ -3643,30 +3610,30 @@
           <t>Priority 1 (Custom Deal)</t>
         </is>
       </c>
-      <c r="H10" s="19" t="n">
+      <c r="H10" s="21" t="n">
         <v>970</v>
       </c>
-      <c r="I10" s="19" t="n">
+      <c r="I10" s="21" t="n">
         <v>30</v>
       </c>
-      <c r="J10" s="20">
+      <c r="J10" s="22">
         <f>H10+I10</f>
         <v/>
       </c>
-      <c r="K10" s="20">
+      <c r="K10" s="22">
         <f>J10*F10</f>
         <v/>
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Mohd Abdul Qadir runs multiple cars. For WagonR, his negotiated rate is ₹970/day. Priority 1 overrides standard slabs. Net daily = ₹970 + ₹30 = ₹1,000. Weekly total for 6 days = ₹6,000.</t>
+          <t>Qadir has a special agreed rate of ₹970/day for his WagonRs. Trips are ignored. Net = ₹970 + ₹30 = ₹1,000/day. Weekly total for 6 days = ₹6,000.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>4B. Multi-Car Operator - Dzire (Mohd Abdul Qadir)</t>
+          <t>4B. Fleet Operator - Dzire (Mohd Abdul Qadir)</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -3695,30 +3662,30 @@
           <t>Priority 1 (Custom Deal)</t>
         </is>
       </c>
-      <c r="H11" s="17" t="n">
+      <c r="H11" s="19" t="n">
         <v>1070</v>
       </c>
-      <c r="I11" s="17" t="n">
+      <c r="I11" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="J11" s="18">
+      <c r="J11" s="20">
         <f>H11+I11</f>
         <v/>
       </c>
-      <c r="K11" s="18">
+      <c r="K11" s="20">
         <f>J11*F11</f>
         <v/>
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>Same operator (Mohd Abdul Qadir) for his Maruti Dzire vehicle. His negotiated deal for Dzire is ₹1,070/day. Net daily = ₹1,070 + ₹30 = ₹1,100. Weekly total for 6 days = ₹6,600. Model rates stay completely separate.</t>
+          <t>For Qadir's Dzire cars, his agreed rate is ₹1,070/day. Net = ₹1,070 + ₹30 = ₹1,100/day. Weekly total for 6 days = ₹6,600. Dzire and WagonR stay separate.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>5. Operator with ₹0 Indemnity (Shaik Kareem)</t>
+          <t>5. Fleet Operator with ₹0 Insurance (Shaik Kareem)</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -3744,33 +3711,33 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>Priority 1 (Custom Deal + ₹0 Indemnity)</t>
-        </is>
-      </c>
-      <c r="H12" s="19" t="n">
+          <t>Priority 1 (Custom Deal + ₹0 Insurance)</t>
+        </is>
+      </c>
+      <c r="H12" s="21" t="n">
         <v>900</v>
       </c>
-      <c r="I12" s="19" t="n">
+      <c r="I12" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="J12" s="20">
+      <c r="J12" s="22">
         <f>H12+I12</f>
         <v/>
       </c>
-      <c r="K12" s="20">
+      <c r="K12" s="22">
         <f>J12*F12</f>
         <v/>
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Shaik Kareem operates Hyundai Xcents in Hyderabad under a custom contract of ₹900/day and ₹0 indemnity. Net daily = ₹900. Weekly total for 5 on-road days = ₹4,500.</t>
+          <t>Shaik Kareem operates Hyundai Xcents under a deal of ₹900/day and ₹0 insurance. Net = ₹900/day. Weekly total for 5 days = ₹4,500.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>6. Maintenance / Workshop Day (Non-Billable)</t>
+          <t>6. Car in Garage / Breakdown</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -3796,26 +3763,26 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Attendance Check: 2 Days Workshop</t>
-        </is>
-      </c>
-      <c r="H13" s="17" t="n">
+          <t>Attendance: 2 Days in Garage</t>
+        </is>
+      </c>
+      <c r="H13" s="19" t="n">
         <v>850</v>
       </c>
-      <c r="I13" s="17" t="n">
+      <c r="I13" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="J13" s="18">
+      <c r="J13" s="20">
         <f>H13+I13</f>
         <v/>
       </c>
-      <c r="K13" s="18">
+      <c r="K13" s="20">
         <f>J13*F13</f>
         <v/>
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>Vehicle was on-road for 4 days and in workshop for 2 days. On workshop days, is_billable_day = FALSE (₹0 rent, ₹0 indemnity). On-road days bill at ₹880/day (75 trips). Weekly total = 4 × ₹880 = ₹3,520.</t>
+          <t>Car was driven 4 days and spent 2 days in the repair shop. On repair days, rent and insurance are ₹0. Only the 4 active days are billed: 4 × ₹880 = ₹3,520.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(rental-spec): clarify priority 2 as the assigned plan from onboarding and remove confusing 2a 2b labels
</commit_message>
<xml_diff>
--- a/Rental Final Table/LetzRyd_Rental_Engine_Master_Specification.xlsx
+++ b/Rental Final Table/LetzRyd_Rental_Engine_Master_Specification.xlsx
@@ -640,12 +640,12 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>This is the official price menu. It lists the daily rent for each trip target (e.g. 50-69 trips) for each city and car model.</t>
+          <t>The official price menu. Lists daily rent for each trip target (e.g. 50-69 trips) and flat rates for each city and car model.</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>The system checks this to find what rent a driver earned from their weekly trips.</t>
+          <t>Used by the system to look up standard rates for drivers.</t>
         </is>
       </c>
     </row>
@@ -667,12 +667,12 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>Lists all drivers and fleet operators, their chosen plan (Uber or All-Platform), and any special discount rates.</t>
+          <t>Lists all drivers and fleet operators, their chosen plan, and any special negotiated rates.</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>The system checks this to see if an operator has a negotiated deal (like ₹970 or ₹1,070/day).</t>
+          <t>Used to check if an operator has a special discount (like ₹970 or ₹1,070/day).</t>
         </is>
       </c>
     </row>
@@ -694,12 +694,12 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>The active contract for each car. It links the car number to the driver, their daily rent, and their daily insurance fee.</t>
+          <t>The active contract for each car. Links car number to the driver, their daily rent, and their daily insurance fee.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>This is the main table the system reads every day to calculate rent.</t>
+          <t>The main table the system reads every day to calculate rent.</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>A permanent history log. Whenever someone changes a car's rent or plan, it records who changed it, when, and why.</t>
+          <t>A permanent history log. Records who changed a car's rent or plan, when, and why.</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -748,7 +748,7 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>The daily bill for each car. Shows if the car was on the road, trips done, daily rent, and daily insurance fee.</t>
+          <t>The daily bill for each car. Shows if the car was driven, weekly trips done, daily rent, and daily insurance fee.</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -760,7 +760,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2. How the Rent is Calculated (Simple Formulas)</t>
+          <t>2. How Rent is Calculated (Simple Formulas)</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
       <c r="C15" s="11" t="n"/>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Calculated for every active car each day. If the car is on the road, both rent and insurance apply. If in garage, both are ₹0.</t>
+          <t>Calculated for every car each day. If the car is on the road, both rent and insurance apply. If in garage, both are ₹0.</t>
         </is>
       </c>
       <c r="E15" s="11" t="n"/>
@@ -816,7 +816,7 @@
       <c r="C17" s="11" t="n"/>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>If a car is broken down or in the workshop, rent is ₹0 and insurance is ₹0 for those days.</t>
+          <t>If a car is in the repair shop, rent is ₹0 and insurance is ₹0 for those days.</t>
         </is>
       </c>
       <c r="E17" s="11" t="n"/>
@@ -841,13 +841,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:F25"/>
+  <dimension ref="A2:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="38" customWidth="1" min="6" max="6"/>
   </cols>
@@ -855,7 +855,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Rental Rules &amp; Step-by-Step Priority Flow</t>
+          <t>Rental Rules &amp; Priority Order</t>
         </is>
       </c>
     </row>
@@ -863,7 +863,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>1. How the System Chooses the Rent (The 3 Priority Steps)</t>
+          <t>1. How the System Decides What Rent to Charge (3 Simple Steps)</t>
         </is>
       </c>
     </row>
@@ -880,17 +880,17 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Question the System Asks</t>
+          <t>Question the System Checks</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>What Happens If YES</t>
+          <t>How the Rent is Decided</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Trip Dependency</t>
+          <t>Trip Requirement</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -908,17 +908,17 @@
       <c r="B7" s="14" t="inlineStr">
         <is>
           <t>Priority 1:
-Special Deal / Custom Agreement</t>
+Special Negotiated Deal</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Does this driver or fleet operator have a negotiated daily rent agreed with LetzRyd?</t>
+          <t>Does this driver or operator have a special agreed rent with LetzRyd?</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>YES: The system charges that agreed rate directly. It stops here. It does not check trip counts or standard rate cards.</t>
+          <t>If YES: The system charges that agreed rate directly. It stops here. It does not look at trips or standard rate cards.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -928,157 +928,163 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Mohd Abdul Qadir: WagonR @ ₹970/day, Dzire @ ₹1,070/day. Shaik Kareem: Xcent @ ₹900/day. Gaadylo: WagonR @ ₹900/day.</t>
+          <t>Mohd Abdul Qadir: WagonR @ ₹970, Dzire @ ₹1,070. Shaik Kareem: Xcent @ ₹900. Gaadylo: WagonR @ ₹900.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>Step 2A</t>
+          <t>Step 2</t>
         </is>
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>Priority 2A:
-Standard All-Platform Plan</t>
+          <t>Priority 2:
+Standard Plan Assigned at Onboarding</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>If no special deal: Is this driver registered on the 'All Platform' plan (allowed to drive for Ola, Rapido, and Uber)?</t>
+          <t>If no special deal: What plan did operations choose for this driver when they were onboarded?
+- Case A: Driver was assigned 'All Platform'
+- Case B: Driver was assigned 'Uber Reducing Rent'</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>YES: The system charges the standard fixed menu rate for that city and car (e.g. ₹1,050 for WagonR, ₹1,200 for Dzire). It stops here.</t>
+          <t>The system checks the driver's assigned plan:
+• If ALL-PLATFORM: Charges the standard flat rate card (₹1,050 for WagonR, ₹1,200 for Dzire).
+• If UBER REDUCING: Counts weekly Uber trips. More trips = lower rent (e.g. 70+ trips drops rent to ₹850).</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>No trips needed. Non-Uber trips are not tracked, so the rate is flat.</t>
+          <t>• All-Platform: No trips needed (rate is flat).
+• Uber Plan: High trip dependency (trips reduce rent).</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>A regular All-Platform driver in Hyderabad or Bangalore pays a flat ₹1,050/day regardless of how many trips they do.</t>
+          <t>• All-Platform: Driver pays flat ₹1,050/day.
+• Uber Plan: Driver doing 75 trips pays ₹850/day instead of ₹1,050 base.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>Step 2B</t>
+          <t>Step 3</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>Priority 2B:
-Standard Uber Reducing Plan</t>
+          <t>Priority 3:
+System Safety Fallback</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>If no special deal: Is this driver on the standard 'Uber Reducing Rent' plan?</t>
+          <t>If no deal and no rate card was found in the sheet (e.g. an unmapped model)?</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>YES: The system counts all Uber trips done from Monday to Sunday. It matches their trip total to the rate card. More trips = lower rent.</t>
+          <t>If YES: The system applies the default model rate (WagonR ₹1,050, Dzire ₹1,200, EC3 ₹1,400) so the system never breaks or charges ₹0 by mistake.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>High trip dependency. Completing more trips moves the driver to a cheaper rate tier.</t>
+          <t>No trips needed. Acts as a safety net.</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>Bangalore WagonR: 0-54 trips = ₹1,050/day. 55-69 trips = ₹950/day. 70+ trips = ₹850/day.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="15" t="inlineStr">
-        <is>
-          <t>Step 3</t>
-        </is>
-      </c>
-      <c r="B10" s="16" t="inlineStr">
-        <is>
-          <t>Priority 3:
-System Fallback Safe Rate</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>If no deal and no matching slab is found in the sheet (e.g. new unmapped model or missing sync)?</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>YES: The system applies the default base rate (WagonR ₹1,050, Dzire ₹1,200, EC3 ₹1,400) so the system never breaks or charges zero.</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>No trips needed. Acts as a safety net.</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>Safely bills the standard base price until operations updates the rate card in the Google Sheet.</t>
+          <t>Safely bills standard base price until operations updates the rate card in the Google Sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2. City-Level Pricing &amp; Insurance Rules</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>2. City-Level Pricing &amp; Insurance Rules</t>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Car Models Used</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Standard Insurance (Indemnity)</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Special Exceptions</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>All-Platform Rate</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>City</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Car Models Used</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Standard Insurance (Indemnity)</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Special Exceptions</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>All-Platform Rate</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Bengaluru (BLR)</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Maruti Wagonr Tour H3 CNG</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>₹30.00 / day</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Nisamudeen K P pays ₹15/day
+Rishad P V pays ₹20/day</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>WagonR: ₹1,050 / day</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Has separate rate tiers for individual drivers vs fleet operators.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>Bengaluru (BLR)</t>
+          <t>Hyderabad (HYD)</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Maruti Wagonr Tour H3 CNG</t>
+          <t>Maruti Wagonr, Maruti Dzire, EC3, Hyundai Xcent (Retired)</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -1088,30 +1094,31 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Nisamudeen K P pays ₹15/day
-Rishad P V pays ₹20/day</t>
+          <t>Retired Hyundai Xcent fleet pays ₹0/day
+Shaik Kareem pays ₹0/day</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>WagonR: ₹1,050 / day</t>
+          <t>WagonR: ₹1,050 / day
+Dzire: ₹1,200 / day</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Has separate rate tiers for individual drivers vs fleet operators.</t>
+          <t>Many fleet operators have negotiated deals that override standard cards.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>Hyderabad (HYD)</t>
+          <t>Mumbai (MUM)</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Maruti Wagonr, Maruti Dzire, EC3, Hyundai Xcent (Retired)</t>
+          <t>Maruti Wagonr Tour H3 CNG</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -1121,166 +1128,132 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Retired Hyundai Xcent fleet pays ₹0/day
-Shaik Kareem pays ₹0/day</t>
+          <t>Added to settlement as 'Insurance Amount'</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>WagonR: ₹1,050 / day
-Dzire: ₹1,200 / day</t>
+          <t>WagonR: ₹1,050 / day</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>Many fleet operators have negotiated deals that override standard cards.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="13" t="inlineStr">
-        <is>
-          <t>Mumbai (MUM)</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Maruti Wagonr Tour H3 CNG</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>₹30.00 / day</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>Added to settlement as 'Insurance Amount'</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>WagonR: ₹1,050 / day</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
           <t>6 trip-reducing tiers starting from 0-49 trips up to 130+ trips.</t>
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>3. Common Operational Situations</t>
+        </is>
+      </c>
+    </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>3. Common Situations &amp; How the System Handles Them</t>
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Situation</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>What Happens in Real Life</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>How the System Handles It</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Result</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Situation</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>What Happens in Real Life</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>How the System Handles It</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Result</t>
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>Operator with Multiple Cars</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>An operator runs both WagonR and Dzire cars.</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Each car has its own record in core_rent. The system matches both the operator ID and the car model.</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Dzires are charged Dzire rent (₹1,070) and WagonRs are charged WagonR rent (₹970). No mixing.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>Operator with Multiple Cars</t>
+          <t>Driver Moonlighting on Ola</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>An operator runs both WagonR and Dzire cars.</t>
+          <t>A driver on the Uber plan spends time driving for Ola.</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Each car has its own record in core_rent. The system matches both the operator ID and the car model.</t>
+          <t>Only Uber trips are counted. Fewer Uber trips mean the driver stays in the lowest tier (0-49 trips).</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Dzires are charged Dzire rent (₹1,070) and WagonRs are charged WagonR rent (₹970). No mixing.</t>
+          <t>Driver pays full base rent (₹1,050/day). The company is fully protected from revenue loss.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>Driver Moonlighting on Ola</t>
+          <t>Mid-Week Plan Change</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>A driver on the Uber plan spends time driving for Ola.</t>
+          <t>A driver wants to switch plans on Wednesday.</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Only Uber trips are counted. Fewer Uber trips mean the driver stays in the lowest tier (0-49 trips).</t>
+          <t>Rent stays locked until Sunday night. Plan changes only take effect starting next Monday.</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Driver pays full base rent (₹1,050/day). The company is fully protected from revenue loss.</t>
+          <t>Stops mid-week recalculation errors and billing disputes with drivers.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>Mid-Week Plan Change</t>
+          <t>Car in Workshop / Breakdown</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>A driver wants to switch plans on Wednesday.</t>
+          <t>A car is in the repair garage for 2 days during the week.</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Rent stays locked until Sunday night. Plan changes only take effect starting next Monday.</t>
+          <t>The daily status is marked 'Maintenance'. The system sets billable = FALSE for those 2 days.</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>Stops mid-week recalculation errors and billing disputes with drivers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
-        <is>
-          <t>Car in Workshop / Breakdown</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>A car is in the repair garage for 2 days during the week.</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>The daily status is marked 'Maintenance'. The system sets billable = FALSE for those 2 days.</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>Driver is charged ₹0 rent and ₹0 insurance for those 2 days.</t>
         </is>
@@ -1333,7 +1306,7 @@
       <c r="A6" s="18" t="inlineStr">
         <is>
           <t>WHAT THIS TABLE IS USED FOR:
-This table is the official price menu copied from the Google Sheet. It stores the weekly trip targets and daily base rents for each city and car model. The system looks at this table to find the rate for standard Uber drivers and standard All-Platform drivers.</t>
+This table stores the official price menu copied from the Google Sheet. It lists the weekly trip targets and daily base rents for each city and car model. The system reads this table to find the rate for standard Uber drivers and standard All-Platform drivers.</t>
         </is>
       </c>
       <c r="B6" s="11" t="n"/>
@@ -3451,7 +3424,7 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Priority 2B (Uber Slab)</t>
+          <t>Priority 2 (Uber Plan)</t>
         </is>
       </c>
       <c r="H7" s="19" t="n">
@@ -3470,7 +3443,7 @@
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>Raju drove exclusively on Uber and did 78 trips. His high trips placed him in the 70+ tier (₹850/day). Net = ₹880/day. Weekly total for 6 days = ₹5,280.</t>
+          <t>Raju was assigned the Uber plan. He completed 78 trips. His high trips earned the 70+ trip tier (₹850/day). Net = ₹880/day. Weekly total for 6 days = ₹5,280.</t>
         </is>
       </c>
     </row>
@@ -3503,7 +3476,7 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>Priority 2B (Uber Tier 1)</t>
+          <t>Priority 2 (Uber Plan)</t>
         </is>
       </c>
       <c r="H8" s="21" t="n">
@@ -3522,7 +3495,7 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Suresh is on an Uber plan but drove for Ola. With only 24 Uber trips recorded, he stays at base price (₹1,050/day). Net = ₹1,080/day. Weekly total = ₹6,480.</t>
+          <t>Suresh was assigned the Uber plan but drove for Ola. With only 24 Uber trips recorded, he stays at base price (₹1,050/day). Net = ₹1,080/day. Weekly total = ₹6,480.</t>
         </is>
       </c>
     </row>
@@ -3555,7 +3528,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Priority 2A (Flat Slab)</t>
+          <t>Priority 2 (All-Platform)</t>
         </is>
       </c>
       <c r="H9" s="19" t="n">
@@ -3574,7 +3547,7 @@
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>Amit drives for Ola, Uber, and Rapido. Trips are not counted. He pays flat menu rent of ₹1,050/day + ₹30 insurance = ₹1,080/day. Weekly total for 7 days = ₹7,560.</t>
+          <t>Amit was assigned All-Platform at onboarding. He pays the flat rate card of ₹1,050/day + ₹30 insurance = ₹1,080/day regardless of how many trips he did.</t>
         </is>
       </c>
     </row>
@@ -3607,7 +3580,7 @@
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>Priority 1 (Custom Deal)</t>
+          <t>Priority 1 (Special Deal)</t>
         </is>
       </c>
       <c r="H10" s="21" t="n">
@@ -3626,7 +3599,7 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Qadir has a special agreed rate of ₹970/day for his WagonRs. Trips are ignored. Net = ₹970 + ₹30 = ₹1,000/day. Weekly total for 6 days = ₹6,000.</t>
+          <t>Qadir has a special agreed deal of ₹970/day for his WagonRs. Trips are ignored. Net = ₹970 + ₹30 = ₹1,000/day. Weekly total for 6 days = ₹6,000.</t>
         </is>
       </c>
     </row>
@@ -3659,7 +3632,7 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Priority 1 (Custom Deal)</t>
+          <t>Priority 1 (Special Deal)</t>
         </is>
       </c>
       <c r="H11" s="19" t="n">
@@ -3678,7 +3651,7 @@
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>For Qadir's Dzire cars, his agreed rate is ₹1,070/day. Net = ₹1,070 + ₹30 = ₹1,100/day. Weekly total for 6 days = ₹6,600. Dzire and WagonR stay separate.</t>
+          <t>For Qadir's Dzire cars, his agreed deal is ₹1,070/day. Net = ₹1,070 + ₹30 = ₹1,100/day. Weekly total for 6 days = ₹6,600. Dzire and WagonR stay separate.</t>
         </is>
       </c>
     </row>
@@ -3711,7 +3684,7 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>Priority 1 (Custom Deal + ₹0 Insurance)</t>
+          <t>Priority 1 (Special Deal + ₹0 Insurance)</t>
         </is>
       </c>
       <c r="H12" s="21" t="n">

</xml_diff>

<commit_message>
docs(rental-spec): clarify priority 2 is vehicle allocation and replace jargon with simple terms
</commit_message>
<xml_diff>
--- a/Rental Final Table/LetzRyd_Rental_Engine_Master_Specification.xlsx
+++ b/Rental Final Table/LetzRyd_Rental_Engine_Master_Specification.xlsx
@@ -684,7 +684,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Created from vehicle assignments</t>
+          <t>Created when a car is assigned (Allocated)</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -844,7 +844,7 @@
   <dimension ref="A2:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
@@ -941,19 +941,18 @@
       <c r="B8" s="16" t="inlineStr">
         <is>
           <t>Priority 2:
-Standard Plan Assigned at Onboarding</t>
+Plan Chosen at Car Allocation (Handover)</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>If no special deal: What plan did operations choose for this driver when they were onboarded?
-- Case A: Driver was assigned 'All Platform'
-- Case B: Driver was assigned 'Uber Reducing Rent'</t>
+          <t>If no special deal: What plan was chosen when the car was handed over (Allocated)?
+*NOTE: If the driver asked for one plan during signup (onboarding) but changed it when picking up the car (allocation), the Allocation plan ALWAYS WINS.</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>The system checks the driver's assigned plan:
+          <t>The system checks the plan selected at allocation:
 • If ALL-PLATFORM: Charges the standard flat rate card (₹1,050 for WagonR, ₹1,200 for Dzire).
 • If UBER REDUCING: Counts weekly Uber trips. More trips = lower rent (e.g. 70+ trips drops rent to ₹850).</t>
         </is>
@@ -1196,12 +1195,12 @@
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>Driver Moonlighting on Ola</t>
+          <t>Driving on Other Apps (Ola or Rapido)</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>A driver on the Uber plan spends time driving for Ola.</t>
+          <t>A driver signed up on the Uber plan spends time taking rides on Ola or Rapido.</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -1211,29 +1210,29 @@
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Driver pays full base rent (₹1,050/day). The company is fully protected from revenue loss.</t>
+          <t>Driver pays full standard rent (₹1,050/day). The company is fully protected from revenue loss.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>Mid-Week Plan Change</t>
+          <t>Switching Plans During Allocation</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>A driver wants to switch plans on Wednesday.</t>
+          <t>Driver chose Uber plan during signup, but switches to All-Platform when picking up the car.</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Rent stays locked until Sunday night. Plan changes only take effect starting next Monday.</t>
+          <t>Allocation record updates core_rent. The system automatically creates an audit record in core_rent_logs.</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Stops mid-week recalculation errors and billing disputes with drivers.</t>
+          <t>Allocation plan wins. Driver gets the All-Platform flat rent immediately.</t>
         </is>
       </c>
     </row>
@@ -2784,7 +2783,7 @@
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>'Driver switched to All-Platform', 'Initial Seed'</t>
+          <t>'Driver switched to All-Platform during allocation', 'Initial Seed'</t>
         </is>
       </c>
     </row>
@@ -3443,14 +3442,14 @@
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>Raju was assigned the Uber plan. He completed 78 trips. His high trips earned the 70+ trip tier (₹850/day). Net = ₹880/day. Weekly total for 6 days = ₹5,280.</t>
+          <t>Raju was allocated the Uber plan. He completed 78 trips. His high trips earned the 70+ trip tier (₹850/day). Net = ₹880/day. Weekly total for 6 days = ₹5,280.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>2. Moonlighting Driver on Ola (Suresh)</t>
+          <t>2. Driving on Other Apps like Ola (Suresh)</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -3495,7 +3494,7 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Suresh was assigned the Uber plan but drove for Ola. With only 24 Uber trips recorded, he stays at base price (₹1,050/day). Net = ₹1,080/day. Weekly total = ₹6,480.</t>
+          <t>Suresh was allocated the Uber plan but took rides on Ola. With only 24 Uber trips recorded, he stays at base price (₹1,050/day). Net = ₹1,080/day. Weekly total = ₹6,480.</t>
         </is>
       </c>
     </row>
@@ -3547,7 +3546,7 @@
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>Amit was assigned All-Platform at onboarding. He pays the flat rate card of ₹1,050/day + ₹30 insurance = ₹1,080/day regardless of how many trips he did.</t>
+          <t>Amit was allocated All-Platform. He pays the flat rate card of ₹1,050/day + ₹30 insurance = ₹1,080/day regardless of how many trips he did.</t>
         </is>
       </c>
     </row>

</xml_diff>